<commit_message>
UK daily ratings for 2026-04-04
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-04-04.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-04-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P141"/>
+  <dimension ref="A1:P190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8712,6 +8712,2928 @@
         <v>0</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>3</v>
+      </c>
+      <c r="G142" t="n">
+        <v>1</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Chasing Time (IRE)</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>3</v>
+      </c>
+      <c r="J142" t="n">
+        <v>133</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="n">
+        <v>160.42</v>
+      </c>
+      <c r="N142" t="n">
+        <v>55</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>3</v>
+      </c>
+      <c r="G143" t="n">
+        <v>2</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Killer Whale (IRE)</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>3</v>
+      </c>
+      <c r="J143" t="n">
+        <v>133</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M143" t="n">
+        <v>160.42</v>
+      </c>
+      <c r="N143" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>3</v>
+      </c>
+      <c r="G144" t="n">
+        <v>3</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Sinocentric</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>3</v>
+      </c>
+      <c r="J144" t="n">
+        <v>133</v>
+      </c>
+      <c r="K144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="M144" t="n">
+        <v>160.42</v>
+      </c>
+      <c r="N144" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>2</v>
+      </c>
+      <c r="C145" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>6</v>
+      </c>
+      <c r="G145" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Coloane (IRE)</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>6</v>
+      </c>
+      <c r="J145" t="n">
+        <v>134</v>
+      </c>
+      <c r="K145" t="n">
+        <v>58</v>
+      </c>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N145" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P145" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>2</v>
+      </c>
+      <c r="C146" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>6</v>
+      </c>
+      <c r="G146" t="n">
+        <v>2</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Book Of Life</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>6</v>
+      </c>
+      <c r="J146" t="n">
+        <v>132</v>
+      </c>
+      <c r="K146" t="n">
+        <v>56</v>
+      </c>
+      <c r="L146" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M146" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N146" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P146" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>2</v>
+      </c>
+      <c r="C147" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>6</v>
+      </c>
+      <c r="G147" t="n">
+        <v>3</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Orbital Chime</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>6</v>
+      </c>
+      <c r="J147" t="n">
+        <v>136</v>
+      </c>
+      <c r="K147" t="n">
+        <v>60</v>
+      </c>
+      <c r="L147" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M147" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N147" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P147" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>2</v>
+      </c>
+      <c r="C148" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>6</v>
+      </c>
+      <c r="G148" t="n">
+        <v>4</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Yehudi (IRE)</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>4</v>
+      </c>
+      <c r="J148" t="n">
+        <v>137</v>
+      </c>
+      <c r="K148" t="n">
+        <v>61</v>
+      </c>
+      <c r="L148" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M148" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N148" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P148" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>2</v>
+      </c>
+      <c r="C149" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>6</v>
+      </c>
+      <c r="G149" t="n">
+        <v>5</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Poetic Force (IRE)</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>12</v>
+      </c>
+      <c r="J149" t="n">
+        <v>140</v>
+      </c>
+      <c r="K149" t="n">
+        <v>64</v>
+      </c>
+      <c r="L149" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="M149" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N149" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P149" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>2</v>
+      </c>
+      <c r="C150" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>6</v>
+      </c>
+      <c r="G150" t="n">
+        <v>6</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Not So Sobers</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>7</v>
+      </c>
+      <c r="J150" t="n">
+        <v>136</v>
+      </c>
+      <c r="K150" t="n">
+        <v>60</v>
+      </c>
+      <c r="L150" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="M150" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N150" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>2</v>
+      </c>
+      <c r="C151" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>6</v>
+      </c>
+      <c r="G151" t="n">
+        <v>7</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Always Fearless (IRE)</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>9</v>
+      </c>
+      <c r="J151" t="n">
+        <v>133</v>
+      </c>
+      <c r="K151" t="n">
+        <v>57</v>
+      </c>
+      <c r="L151" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="M151" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N151" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>2</v>
+      </c>
+      <c r="C152" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>6</v>
+      </c>
+      <c r="G152" t="n">
+        <v>8</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Nala The Lioness</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>6</v>
+      </c>
+      <c r="J152" t="n">
+        <v>129</v>
+      </c>
+      <c r="K152" t="n">
+        <v>53</v>
+      </c>
+      <c r="L152" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="M152" t="n">
+        <v>114.66</v>
+      </c>
+      <c r="N152" t="n">
+        <v>-33.7</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>4</v>
+      </c>
+      <c r="G153" t="n">
+        <v>1</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Constant Star (IRE)</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>3</v>
+      </c>
+      <c r="J153" t="n">
+        <v>128</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N153" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>3</v>
+      </c>
+      <c r="C154" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>4</v>
+      </c>
+      <c r="G154" t="n">
+        <v>2</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Imelda (IRE)</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>3</v>
+      </c>
+      <c r="J154" t="n">
+        <v>124</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="M154" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N154" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P154" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>3</v>
+      </c>
+      <c r="C155" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>4</v>
+      </c>
+      <c r="G155" t="n">
+        <v>3</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Safe Zone (IRE)</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>3</v>
+      </c>
+      <c r="J155" t="n">
+        <v>128</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="M155" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N155" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>3</v>
+      </c>
+      <c r="C156" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>4</v>
+      </c>
+      <c r="G156" t="n">
+        <v>4</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Thimble</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>3</v>
+      </c>
+      <c r="J156" t="n">
+        <v>126</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="M156" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N156" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P156" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>3</v>
+      </c>
+      <c r="C157" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>4</v>
+      </c>
+      <c r="G157" t="n">
+        <v>5</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Rogue Desire (FR)</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>3</v>
+      </c>
+      <c r="J157" t="n">
+        <v>128</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="M157" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N157" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>3</v>
+      </c>
+      <c r="C158" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>4</v>
+      </c>
+      <c r="G158" t="n">
+        <v>6</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Thai Princess</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>3</v>
+      </c>
+      <c r="J158" t="n">
+        <v>126</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="M158" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N158" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>3</v>
+      </c>
+      <c r="C159" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>4</v>
+      </c>
+      <c r="G159" t="n">
+        <v>7</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Difford Girl</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>4</v>
+      </c>
+      <c r="J159" t="n">
+        <v>140</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="M159" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N159" t="n">
+        <v>-14.9</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>3</v>
+      </c>
+      <c r="C160" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>4</v>
+      </c>
+      <c r="G160" t="n">
+        <v>8</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Action Reaction</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>3</v>
+      </c>
+      <c r="J160" t="n">
+        <v>124</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="M160" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="N160" t="n">
+        <v>-36.9</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>4</v>
+      </c>
+      <c r="C161" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>5</v>
+      </c>
+      <c r="G161" t="n">
+        <v>1</v>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Kirkdale (IRE)</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>4</v>
+      </c>
+      <c r="J161" t="n">
+        <v>135</v>
+      </c>
+      <c r="K161" t="n">
+        <v>70</v>
+      </c>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N161" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>4</v>
+      </c>
+      <c r="C162" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>5</v>
+      </c>
+      <c r="G162" t="n">
+        <v>2</v>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Lequinto (IRE)</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>9</v>
+      </c>
+      <c r="J162" t="n">
+        <v>133</v>
+      </c>
+      <c r="K162" t="n">
+        <v>68</v>
+      </c>
+      <c r="L162" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M162" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N162" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>4</v>
+      </c>
+      <c r="C163" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>5</v>
+      </c>
+      <c r="G163" t="n">
+        <v>3</v>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Punchbowl Flyer (IRE)</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>9</v>
+      </c>
+      <c r="J163" t="n">
+        <v>126</v>
+      </c>
+      <c r="K163" t="n">
+        <v>61</v>
+      </c>
+      <c r="L163" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="M163" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N163" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>4</v>
+      </c>
+      <c r="C164" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>5</v>
+      </c>
+      <c r="G164" t="n">
+        <v>4</v>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Valsharah (IRE)</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>4</v>
+      </c>
+      <c r="J164" t="n">
+        <v>122</v>
+      </c>
+      <c r="K164" t="n">
+        <v>57</v>
+      </c>
+      <c r="L164" t="n">
+        <v>3</v>
+      </c>
+      <c r="M164" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N164" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P164" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>4</v>
+      </c>
+      <c r="C165" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>5</v>
+      </c>
+      <c r="G165" t="n">
+        <v>5</v>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Cayman Tai (IRE)</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>4</v>
+      </c>
+      <c r="J165" t="n">
+        <v>135</v>
+      </c>
+      <c r="K165" t="n">
+        <v>70</v>
+      </c>
+      <c r="L165" t="n">
+        <v>4</v>
+      </c>
+      <c r="M165" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N165" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P165" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>4</v>
+      </c>
+      <c r="C166" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>5</v>
+      </c>
+      <c r="G166" t="n">
+        <v>6</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Pianoforte</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>5</v>
+      </c>
+      <c r="J166" t="n">
+        <v>132</v>
+      </c>
+      <c r="K166" t="n">
+        <v>67</v>
+      </c>
+      <c r="L166" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M166" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N166" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>4</v>
+      </c>
+      <c r="C167" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>5</v>
+      </c>
+      <c r="G167" t="n">
+        <v>7</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>6</v>
+      </c>
+      <c r="J167" t="n">
+        <v>127</v>
+      </c>
+      <c r="K167" t="n">
+        <v>62</v>
+      </c>
+      <c r="L167" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="M167" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N167" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>4</v>
+      </c>
+      <c r="C168" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>5</v>
+      </c>
+      <c r="G168" t="n">
+        <v>8</v>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Brian The Snail (IRE)</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>12</v>
+      </c>
+      <c r="J168" t="n">
+        <v>126</v>
+      </c>
+      <c r="K168" t="n">
+        <v>61</v>
+      </c>
+      <c r="L168" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="M168" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N168" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>4</v>
+      </c>
+      <c r="C169" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>5</v>
+      </c>
+      <c r="G169" t="n">
+        <v>9</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Megaphone</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>4</v>
+      </c>
+      <c r="J169" t="n">
+        <v>125</v>
+      </c>
+      <c r="K169" t="n">
+        <v>60</v>
+      </c>
+      <c r="L169" t="n">
+        <v>10</v>
+      </c>
+      <c r="M169" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="N169" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>5</v>
+      </c>
+      <c r="C170" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>4</v>
+      </c>
+      <c r="G170" t="n">
+        <v>1</v>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Pride Of Donegal (IRE)</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>4</v>
+      </c>
+      <c r="J170" t="n">
+        <v>134</v>
+      </c>
+      <c r="K170" t="n">
+        <v>84</v>
+      </c>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N170" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P170" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>5</v>
+      </c>
+      <c r="C171" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>4</v>
+      </c>
+      <c r="G171" t="n">
+        <v>2</v>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Charmaine</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>5</v>
+      </c>
+      <c r="J171" t="n">
+        <v>136</v>
+      </c>
+      <c r="K171" t="n">
+        <v>86</v>
+      </c>
+      <c r="L171" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="M171" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N171" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>5</v>
+      </c>
+      <c r="C172" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>4</v>
+      </c>
+      <c r="G172" t="n">
+        <v>3</v>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Codiak (IRE)</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>4</v>
+      </c>
+      <c r="J172" t="n">
+        <v>134</v>
+      </c>
+      <c r="K172" t="n">
+        <v>84</v>
+      </c>
+      <c r="L172" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="M172" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N172" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>5</v>
+      </c>
+      <c r="C173" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>4</v>
+      </c>
+      <c r="G173" t="n">
+        <v>4</v>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Maasai Mara</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>6</v>
+      </c>
+      <c r="J173" t="n">
+        <v>128</v>
+      </c>
+      <c r="K173" t="n">
+        <v>78</v>
+      </c>
+      <c r="L173" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="M173" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N173" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>5</v>
+      </c>
+      <c r="C174" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>4</v>
+      </c>
+      <c r="G174" t="n">
+        <v>5</v>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Gemmari</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>4</v>
+      </c>
+      <c r="J174" t="n">
+        <v>126</v>
+      </c>
+      <c r="K174" t="n">
+        <v>76</v>
+      </c>
+      <c r="L174" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="M174" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N174" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P174" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>5</v>
+      </c>
+      <c r="C175" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>4</v>
+      </c>
+      <c r="G175" t="n">
+        <v>6</v>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Bulldog Spirit (IRE)</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>6</v>
+      </c>
+      <c r="J175" t="n">
+        <v>122</v>
+      </c>
+      <c r="K175" t="n">
+        <v>72</v>
+      </c>
+      <c r="L175" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="M175" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N175" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>5</v>
+      </c>
+      <c r="C176" t="n">
+        <v>12.23181818181818</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>4</v>
+      </c>
+      <c r="G176" t="n">
+        <v>7</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Polling Day (IRE)</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>8</v>
+      </c>
+      <c r="J176" t="n">
+        <v>126</v>
+      </c>
+      <c r="K176" t="n">
+        <v>76</v>
+      </c>
+      <c r="L176" t="n">
+        <v>17.25</v>
+      </c>
+      <c r="M176" t="n">
+        <v>159.95</v>
+      </c>
+      <c r="N176" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P176" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>6</v>
+      </c>
+      <c r="C177" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>5</v>
+      </c>
+      <c r="G177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Betweenthesticks</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>6</v>
+      </c>
+      <c r="J177" t="n">
+        <v>134</v>
+      </c>
+      <c r="K177" t="n">
+        <v>66</v>
+      </c>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N177" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P177" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>6</v>
+      </c>
+      <c r="C178" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>5</v>
+      </c>
+      <c r="G178" t="n">
+        <v>2</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Shalaa Asker</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>8</v>
+      </c>
+      <c r="J178" t="n">
+        <v>135</v>
+      </c>
+      <c r="K178" t="n">
+        <v>67</v>
+      </c>
+      <c r="L178" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M178" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N178" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P178" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>6</v>
+      </c>
+      <c r="C179" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>5</v>
+      </c>
+      <c r="G179" t="n">
+        <v>3</v>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Blue Force (IRE)</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>5</v>
+      </c>
+      <c r="J179" t="n">
+        <v>133</v>
+      </c>
+      <c r="K179" t="n">
+        <v>65</v>
+      </c>
+      <c r="L179" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="M179" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N179" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>6</v>
+      </c>
+      <c r="C180" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>5</v>
+      </c>
+      <c r="G180" t="n">
+        <v>4</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Candy Warhol (USA)</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>7</v>
+      </c>
+      <c r="J180" t="n">
+        <v>128</v>
+      </c>
+      <c r="K180" t="n">
+        <v>60</v>
+      </c>
+      <c r="L180" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M180" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N180" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P180" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>6</v>
+      </c>
+      <c r="C181" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>5</v>
+      </c>
+      <c r="G181" t="n">
+        <v>5</v>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Phoenix Beach (IRE)</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>7</v>
+      </c>
+      <c r="J181" t="n">
+        <v>126</v>
+      </c>
+      <c r="K181" t="n">
+        <v>58</v>
+      </c>
+      <c r="L181" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="M181" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N181" t="n">
+        <v>49</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P181" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>6</v>
+      </c>
+      <c r="C182" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>5</v>
+      </c>
+      <c r="G182" t="n">
+        <v>6</v>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Beaming Light</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>6</v>
+      </c>
+      <c r="J182" t="n">
+        <v>132</v>
+      </c>
+      <c r="K182" t="n">
+        <v>64</v>
+      </c>
+      <c r="L182" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M182" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N182" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>6</v>
+      </c>
+      <c r="C183" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>5</v>
+      </c>
+      <c r="G183" t="n">
+        <v>7</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Amerjeet</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>4</v>
+      </c>
+      <c r="J183" t="n">
+        <v>123</v>
+      </c>
+      <c r="K183" t="n">
+        <v>55</v>
+      </c>
+      <c r="L183" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="M183" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N183" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P183" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>6</v>
+      </c>
+      <c r="C184" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>5</v>
+      </c>
+      <c r="G184" t="n">
+        <v>8</v>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Toomuchforme</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>4</v>
+      </c>
+      <c r="J184" t="n">
+        <v>135</v>
+      </c>
+      <c r="K184" t="n">
+        <v>67</v>
+      </c>
+      <c r="L184" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="M184" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="N184" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P184" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>7</v>
+      </c>
+      <c r="C185" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>6</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Raspoutine</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>3</v>
+      </c>
+      <c r="J185" t="n">
+        <v>135</v>
+      </c>
+      <c r="K185" t="n">
+        <v>60</v>
+      </c>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P185" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>7</v>
+      </c>
+      <c r="C186" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>6</v>
+      </c>
+      <c r="G186" t="n">
+        <v>1</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Karakula Dancer</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>3</v>
+      </c>
+      <c r="J186" t="n">
+        <v>134</v>
+      </c>
+      <c r="K186" t="n">
+        <v>59</v>
+      </c>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N186" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P186" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>7</v>
+      </c>
+      <c r="C187" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>6</v>
+      </c>
+      <c r="G187" t="n">
+        <v>2</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Lexington Express (IRE)</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>3</v>
+      </c>
+      <c r="J187" t="n">
+        <v>138</v>
+      </c>
+      <c r="K187" t="n">
+        <v>63</v>
+      </c>
+      <c r="L187" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M187" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N187" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P187" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>7</v>
+      </c>
+      <c r="C188" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>6</v>
+      </c>
+      <c r="G188" t="n">
+        <v>3</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Zoustellar (IRE)</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>3</v>
+      </c>
+      <c r="J188" t="n">
+        <v>132</v>
+      </c>
+      <c r="K188" t="n">
+        <v>57</v>
+      </c>
+      <c r="L188" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M188" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N188" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P188" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>7</v>
+      </c>
+      <c r="C189" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>6</v>
+      </c>
+      <c r="G189" t="n">
+        <v>4</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Panthere Noir</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>3</v>
+      </c>
+      <c r="J189" t="n">
+        <v>128</v>
+      </c>
+      <c r="K189" t="n">
+        <v>53</v>
+      </c>
+      <c r="L189" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="M189" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N189" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P189" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>7</v>
+      </c>
+      <c r="C190" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>6</v>
+      </c>
+      <c r="G190" t="n">
+        <v>5</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Amazing Anita</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>3</v>
+      </c>
+      <c r="J190" t="n">
+        <v>135</v>
+      </c>
+      <c r="K190" t="n">
+        <v>60</v>
+      </c>
+      <c r="L190" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="M190" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="N190" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P190" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>